<commit_message>
Audit and harden all 10 GitHub Actions workflows for 100% successful execution
</commit_message>
<xml_diff>
--- a/Test_Results/Backend_Report.xlsx
+++ b/Test_Results/Backend_Report.xlsx
@@ -525,7 +525,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0055</v>
+        <v>0.0075</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -555,7 +555,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0024</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -585,7 +585,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.0021</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0041</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -645,7 +645,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0043</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -675,7 +675,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0048</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -735,7 +735,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0029</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -765,7 +765,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0027</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -795,7 +795,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.004</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -825,7 +825,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0028</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -855,7 +855,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0021</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -885,7 +885,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -915,7 +915,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0069</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -945,7 +945,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.003</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -975,7 +975,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.003</v>
+        <v>0.0075</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -1005,7 +1005,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0043</v>
+        <v>0.0067</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -1035,7 +1035,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.0185</v>
+        <v>0.0148</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0154</v>
+        <v>0.0166</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -1095,7 +1095,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0036</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -1125,7 +1125,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.005</v>
+        <v>0.0029</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -1185,7 +1185,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.018</v>
+        <v>0.02</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -1215,7 +1215,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0033</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -1245,7 +1245,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.0218</v>
+        <v>0.0251</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -1275,7 +1275,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0026</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -1305,7 +1305,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0028</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -1335,7 +1335,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.024</v>
+        <v>0.019</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -1365,7 +1365,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.012</v>
+        <v>0.0116</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -1395,7 +1395,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0011</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -1425,7 +1425,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0181</v>
+        <v>0.0175</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -1455,7 +1455,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0172</v>
+        <v>0.0156</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -1485,7 +1485,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.0164</v>
+        <v>0.0081</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -1515,7 +1515,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.0128</v>
+        <v>0.0098</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -1545,7 +1545,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0012</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -1575,7 +1575,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0046</v>
+        <v>0.0037</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -1605,7 +1605,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0018</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -1635,7 +1635,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0021</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.0095</v>
+        <v>0.0072</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0012</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -1725,7 +1725,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.003</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -1755,7 +1755,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0222</v>
+        <v>0.0206</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -1785,7 +1785,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.0036</v>
+        <v>0.004</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -1815,7 +1815,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0021</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.002</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -1875,7 +1875,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0018</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -1905,7 +1905,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0027</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -1965,7 +1965,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.0054</v>
+        <v>0.0136</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -1995,7 +1995,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0027</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0013</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -2055,7 +2055,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.0101</v>
+        <v>0.0074</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -2085,7 +2085,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.0013</v>
+        <v>0.0021</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0026</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -2199,7 +2199,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0016</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -2229,7 +2229,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.0013</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -2259,7 +2259,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0016</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -2289,7 +2289,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.0026</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -2319,7 +2319,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0017</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0019</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -2379,7 +2379,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0068</v>
+        <v>0.0078</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -2409,7 +2409,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0011</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -2439,7 +2439,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.001</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -2499,7 +2499,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0013</v>
+        <v>0.0018</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0011</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -2559,7 +2559,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0026</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -2589,7 +2589,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.1892</v>
+        <v>0.1765</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -2619,7 +2619,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.002</v>
+        <v>0.001</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -2649,7 +2649,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0009</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -2679,7 +2679,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0009</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -2709,7 +2709,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.2178</v>
+        <v>0.1734</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -2739,7 +2739,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.2317</v>
+        <v>0.2018</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -2769,7 +2769,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.2473</v>
+        <v>0.1711</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -2799,7 +2799,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.2511</v>
+        <v>0.1699</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -2829,7 +2829,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.2461</v>
+        <v>0.1647</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -2859,7 +2859,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0024</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -2889,7 +2889,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0131</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -2919,7 +2919,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.0055</v>
+        <v>0.0021</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -2949,7 +2949,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.002</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -2979,7 +2979,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.3121</v>
+        <v>0.1587</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -3009,7 +3009,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0051</v>
+        <v>0.0021</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -3039,7 +3039,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0042</v>
+        <v>0.0036</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -3069,7 +3069,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0018</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -3099,7 +3099,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.3276</v>
+        <v>0.1539</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -3129,7 +3129,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0074</v>
+        <v>0.0042</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -3159,7 +3159,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0016</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -3189,7 +3189,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.003</v>
+        <v>0.0015</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -3219,7 +3219,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.0048</v>
+        <v>0.0018</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -3249,7 +3249,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0042</v>
+        <v>0.0029</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -3279,7 +3279,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0024</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -3309,7 +3309,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.0044</v>
+        <v>0.0019</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -3339,7 +3339,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0037</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -3369,7 +3369,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.0045</v>
+        <v>0.003</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -3399,7 +3399,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0042</v>
+        <v>0.0023</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -3429,7 +3429,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0016</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -3459,7 +3459,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0017</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -3489,7 +3489,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0015</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -3573,7 +3573,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0121</v>
+        <v>0.0119</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -3603,7 +3603,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0014</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -3633,7 +3633,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.0109</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -3663,7 +3663,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0227</v>
+        <v>0.0178</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -3693,7 +3693,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0407</v>
+        <v>0.0329</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -3723,7 +3723,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0113</v>
+        <v>0.0121</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -3753,7 +3753,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.01</v>
+        <v>0.0135</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -3783,7 +3783,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0031</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.0013</v>
+        <v>0.0017</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -3873,7 +3873,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0156</v>
+        <v>0.022</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -3903,7 +3903,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0022</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -3933,7 +3933,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0094</v>
+        <v>0.0127</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -3963,7 +3963,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.0173</v>
+        <v>0.0157</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -3993,7 +3993,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.0242</v>
+        <v>0.03</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -4023,7 +4023,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.0359</v>
+        <v>0.0309</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -4053,7 +4053,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0073</v>
+        <v>0.0059</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -4083,7 +4083,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.0186</v>
+        <v>0.0174</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -4113,7 +4113,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.008999999999999999</v>
+        <v>0.009299999999999999</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -4143,7 +4143,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0127</v>
+        <v>0.0133</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -4173,7 +4173,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.0013</v>
+        <v>0.0024</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -4203,7 +4203,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.002</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -4233,7 +4233,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.002</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -4263,7 +4263,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0037</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -4293,7 +4293,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0031</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -4323,7 +4323,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0054</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -4353,7 +4353,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.007</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0033</v>
+        <v>0.0045</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -4413,7 +4413,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0045</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -4443,7 +4443,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.005</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -4473,7 +4473,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0063</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -4503,7 +4503,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.005</v>
+        <v>0.0041</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -4533,7 +4533,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0016</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0035</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -4593,7 +4593,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0026</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -4623,7 +4623,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0022</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -4653,7 +4653,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0042</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -4683,7 +4683,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0016</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -4713,7 +4713,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0046</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0032</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -4773,7 +4773,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0113</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -4803,7 +4803,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0047</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -4833,7 +4833,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.003</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -4863,7 +4863,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.003</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -4893,7 +4893,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0041</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -4923,7 +4923,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.003</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -4953,7 +4953,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0021</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -4983,7 +4983,7 @@
         </is>
       </c>
       <c r="E49" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.0044</v>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
@@ -5013,7 +5013,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0027</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -5043,7 +5043,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>1.1962</v>
+        <v>1.4947</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -5073,7 +5073,7 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0041</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0034</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -5133,7 +5133,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0035</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -5163,7 +5163,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0032</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -5193,7 +5193,7 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0032</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -5223,7 +5223,7 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0021</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -5253,7 +5253,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0025</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -5283,7 +5283,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0018</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -5313,7 +5313,7 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.002</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -5343,7 +5343,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.0114</v>
+        <v>0.0089</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -5373,7 +5373,7 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.2659</v>
+        <v>0.264</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -5433,7 +5433,7 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.002</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -5463,7 +5463,7 @@
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.0332</v>
+        <v>0.0404</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -5547,7 +5547,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.1901</v>
+        <v>0.2167</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -5607,7 +5607,7 @@
         </is>
       </c>
       <c r="E4" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0018</v>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
@@ -5637,7 +5637,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.5318000000000001</v>
+        <v>0.6742</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -5667,7 +5667,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.188</v>
+        <v>0.2264</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -5697,7 +5697,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.2195</v>
+        <v>0.2479</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -5727,7 +5727,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.002</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -5757,7 +5757,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0015</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -5787,7 +5787,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.002</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -5817,7 +5817,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0019</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -5847,7 +5847,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.0075</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -5877,7 +5877,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.2564</v>
+        <v>0.2025</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -5907,7 +5907,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0015</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -5937,7 +5937,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0025</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -5967,7 +5967,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.0044</v>
+        <v>0.0073</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -5997,7 +5997,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0049</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -6027,7 +6027,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0075</v>
+        <v>0.0038</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -6057,7 +6057,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0019</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -6087,7 +6087,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0011</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -6117,7 +6117,7 @@
         </is>
       </c>
       <c r="E21" s="2" t="n">
-        <v>0.0041</v>
+        <v>0.0033</v>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
@@ -6147,7 +6147,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.0104</v>
+        <v>0.0078</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -6177,7 +6177,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.0047</v>
+        <v>0.0013</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -6207,7 +6207,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0281</v>
+        <v>0.0192</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -6237,7 +6237,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0232</v>
+        <v>0.021</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -6267,7 +6267,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0012</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -6297,7 +6297,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0049</v>
+        <v>0.0024</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -6327,7 +6327,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0051</v>
+        <v>0.0026</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -6357,7 +6357,7 @@
         </is>
       </c>
       <c r="E29" s="2" t="n">
-        <v>0.0044</v>
+        <v>0.0019</v>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
@@ -6387,7 +6387,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0291</v>
+        <v>0.0294</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -6471,7 +6471,7 @@
         </is>
       </c>
       <c r="E2" s="2" t="n">
-        <v>0.0054</v>
+        <v>0.0058</v>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
@@ -6501,7 +6501,7 @@
         </is>
       </c>
       <c r="E3" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0044</v>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
@@ -6561,7 +6561,7 @@
         </is>
       </c>
       <c r="E5" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0041</v>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
@@ -6591,7 +6591,7 @@
         </is>
       </c>
       <c r="E6" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0123</v>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
@@ -6621,7 +6621,7 @@
         </is>
       </c>
       <c r="E7" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0078</v>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
@@ -6651,7 +6651,7 @@
         </is>
       </c>
       <c r="E8" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0052</v>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
@@ -6681,7 +6681,7 @@
         </is>
       </c>
       <c r="E9" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0386</v>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
@@ -6711,7 +6711,7 @@
         </is>
       </c>
       <c r="E10" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0073</v>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
@@ -6741,7 +6741,7 @@
         </is>
       </c>
       <c r="E11" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0069</v>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
@@ -6771,7 +6771,7 @@
         </is>
       </c>
       <c r="E12" s="2" t="n">
-        <v>0.003</v>
+        <v>0.025</v>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
@@ -6801,7 +6801,7 @@
         </is>
       </c>
       <c r="E13" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0043</v>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
@@ -6831,7 +6831,7 @@
         </is>
       </c>
       <c r="E14" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0048</v>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
@@ -6861,7 +6861,7 @@
         </is>
       </c>
       <c r="E15" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.0041</v>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
@@ -6891,7 +6891,7 @@
         </is>
       </c>
       <c r="E16" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0025</v>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
@@ -6921,7 +6921,7 @@
         </is>
       </c>
       <c r="E17" s="2" t="n">
-        <v>0.002</v>
+        <v>0.008</v>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
@@ -6951,7 +6951,7 @@
         </is>
       </c>
       <c r="E18" s="2" t="n">
-        <v>0.0033</v>
+        <v>0.0071</v>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
@@ -6981,7 +6981,7 @@
         </is>
       </c>
       <c r="E19" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0032</v>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
@@ -7011,7 +7011,7 @@
         </is>
       </c>
       <c r="E20" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0026</v>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
@@ -7071,7 +7071,7 @@
         </is>
       </c>
       <c r="E22" s="2" t="n">
-        <v>0.0036</v>
+        <v>0.0024</v>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
@@ -7101,7 +7101,7 @@
         </is>
       </c>
       <c r="E23" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0024</v>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
@@ -7131,7 +7131,7 @@
         </is>
       </c>
       <c r="E24" s="2" t="n">
-        <v>0.0148</v>
+        <v>0.004</v>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
@@ -7161,7 +7161,7 @@
         </is>
       </c>
       <c r="E25" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0043</v>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
@@ -7191,7 +7191,7 @@
         </is>
       </c>
       <c r="E26" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0023</v>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
@@ -7221,7 +7221,7 @@
         </is>
       </c>
       <c r="E27" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0022</v>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
@@ -7251,7 +7251,7 @@
         </is>
       </c>
       <c r="E28" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0041</v>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
@@ -7311,7 +7311,7 @@
         </is>
       </c>
       <c r="E30" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0029</v>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
@@ -7341,7 +7341,7 @@
         </is>
       </c>
       <c r="E31" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.004</v>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
@@ -7371,7 +7371,7 @@
         </is>
       </c>
       <c r="E32" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0022</v>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
@@ -7401,7 +7401,7 @@
         </is>
       </c>
       <c r="E33" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0021</v>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
@@ -7431,7 +7431,7 @@
         </is>
       </c>
       <c r="E34" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0023</v>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
@@ -7461,7 +7461,7 @@
         </is>
       </c>
       <c r="E35" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0024</v>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
@@ -7491,7 +7491,7 @@
         </is>
       </c>
       <c r="E36" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0022</v>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
@@ -7521,7 +7521,7 @@
         </is>
       </c>
       <c r="E37" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.002</v>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
@@ -7551,7 +7551,7 @@
         </is>
       </c>
       <c r="E38" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0027</v>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
@@ -7581,7 +7581,7 @@
         </is>
       </c>
       <c r="E39" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0022</v>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
@@ -7611,7 +7611,7 @@
         </is>
       </c>
       <c r="E40" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0025</v>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
@@ -7641,7 +7641,7 @@
         </is>
       </c>
       <c r="E41" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.002</v>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
@@ -7671,7 +7671,7 @@
         </is>
       </c>
       <c r="E42" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0024</v>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
@@ -7701,7 +7701,7 @@
         </is>
       </c>
       <c r="E43" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.002</v>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
@@ -7731,7 +7731,7 @@
         </is>
       </c>
       <c r="E44" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.003</v>
       </c>
       <c r="F44" s="2" t="inlineStr">
         <is>
@@ -7761,7 +7761,7 @@
         </is>
       </c>
       <c r="E45" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0022</v>
       </c>
       <c r="F45" s="2" t="inlineStr">
         <is>
@@ -7791,7 +7791,7 @@
         </is>
       </c>
       <c r="E46" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0029</v>
       </c>
       <c r="F46" s="2" t="inlineStr">
         <is>
@@ -7821,7 +7821,7 @@
         </is>
       </c>
       <c r="E47" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0022</v>
       </c>
       <c r="F47" s="2" t="inlineStr">
         <is>
@@ -7851,7 +7851,7 @@
         </is>
       </c>
       <c r="E48" s="2" t="n">
-        <v>0.003</v>
+        <v>0.002</v>
       </c>
       <c r="F48" s="2" t="inlineStr">
         <is>
@@ -7911,7 +7911,7 @@
         </is>
       </c>
       <c r="E50" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0035</v>
       </c>
       <c r="F50" s="2" t="inlineStr">
         <is>
@@ -7941,7 +7941,7 @@
         </is>
       </c>
       <c r="E51" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0022</v>
       </c>
       <c r="F51" s="2" t="inlineStr">
         <is>
@@ -7971,7 +7971,7 @@
         </is>
       </c>
       <c r="E52" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0025</v>
       </c>
       <c r="F52" s="2" t="inlineStr">
         <is>
@@ -8001,7 +8001,7 @@
         </is>
       </c>
       <c r="E53" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0023</v>
       </c>
       <c r="F53" s="2" t="inlineStr">
         <is>
@@ -8031,7 +8031,7 @@
         </is>
       </c>
       <c r="E54" s="2" t="n">
-        <v>0.0042</v>
+        <v>0.0021</v>
       </c>
       <c r="F54" s="2" t="inlineStr">
         <is>
@@ -8061,7 +8061,7 @@
         </is>
       </c>
       <c r="E55" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0021</v>
       </c>
       <c r="F55" s="2" t="inlineStr">
         <is>
@@ -8091,7 +8091,7 @@
         </is>
       </c>
       <c r="E56" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.0021</v>
       </c>
       <c r="F56" s="2" t="inlineStr">
         <is>
@@ -8121,7 +8121,7 @@
         </is>
       </c>
       <c r="E57" s="2" t="n">
-        <v>0.0033</v>
+        <v>0.0022</v>
       </c>
       <c r="F57" s="2" t="inlineStr">
         <is>
@@ -8151,7 +8151,7 @@
         </is>
       </c>
       <c r="E58" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.002</v>
       </c>
       <c r="F58" s="2" t="inlineStr">
         <is>
@@ -8181,7 +8181,7 @@
         </is>
       </c>
       <c r="E59" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0024</v>
       </c>
       <c r="F59" s="2" t="inlineStr">
         <is>
@@ -8211,7 +8211,7 @@
         </is>
       </c>
       <c r="E60" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.002</v>
       </c>
       <c r="F60" s="2" t="inlineStr">
         <is>
@@ -8241,7 +8241,7 @@
         </is>
       </c>
       <c r="E61" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0019</v>
       </c>
       <c r="F61" s="2" t="inlineStr">
         <is>
@@ -8271,7 +8271,7 @@
         </is>
       </c>
       <c r="E62" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.002</v>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
@@ -8301,7 +8301,7 @@
         </is>
       </c>
       <c r="E63" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0038</v>
       </c>
       <c r="F63" s="2" t="inlineStr">
         <is>
@@ -8331,7 +8331,7 @@
         </is>
       </c>
       <c r="E64" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0033</v>
       </c>
       <c r="F64" s="2" t="inlineStr">
         <is>
@@ -8361,7 +8361,7 @@
         </is>
       </c>
       <c r="E65" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0021</v>
       </c>
       <c r="F65" s="2" t="inlineStr">
         <is>
@@ -8391,7 +8391,7 @@
         </is>
       </c>
       <c r="E66" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0021</v>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
@@ -8421,7 +8421,7 @@
         </is>
       </c>
       <c r="E67" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0039</v>
       </c>
       <c r="F67" s="2" t="inlineStr">
         <is>
@@ -8451,7 +8451,7 @@
         </is>
       </c>
       <c r="E68" s="2" t="n">
-        <v>0.0033</v>
+        <v>0.0029</v>
       </c>
       <c r="F68" s="2" t="inlineStr">
         <is>
@@ -8481,7 +8481,7 @@
         </is>
       </c>
       <c r="E69" s="2" t="n">
-        <v>0.0044</v>
+        <v>0.0028</v>
       </c>
       <c r="F69" s="2" t="inlineStr">
         <is>
@@ -8511,7 +8511,7 @@
         </is>
       </c>
       <c r="E70" s="2" t="n">
-        <v>0.0034</v>
+        <v>0.0043</v>
       </c>
       <c r="F70" s="2" t="inlineStr">
         <is>
@@ -8541,7 +8541,7 @@
         </is>
       </c>
       <c r="E71" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0021</v>
       </c>
       <c r="F71" s="2" t="inlineStr">
         <is>
@@ -8571,7 +8571,7 @@
         </is>
       </c>
       <c r="E72" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0021</v>
       </c>
       <c r="F72" s="2" t="inlineStr">
         <is>
@@ -8601,7 +8601,7 @@
         </is>
       </c>
       <c r="E73" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0022</v>
       </c>
       <c r="F73" s="2" t="inlineStr">
         <is>
@@ -8631,7 +8631,7 @@
         </is>
       </c>
       <c r="E74" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0039</v>
       </c>
       <c r="F74" s="2" t="inlineStr">
         <is>
@@ -8661,7 +8661,7 @@
         </is>
       </c>
       <c r="E75" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0184</v>
       </c>
       <c r="F75" s="2" t="inlineStr">
         <is>
@@ -8691,7 +8691,7 @@
         </is>
       </c>
       <c r="E76" s="2" t="n">
-        <v>0.0036</v>
+        <v>0.0029</v>
       </c>
       <c r="F76" s="2" t="inlineStr">
         <is>
@@ -8721,7 +8721,7 @@
         </is>
       </c>
       <c r="E77" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0026</v>
       </c>
       <c r="F77" s="2" t="inlineStr">
         <is>
@@ -8751,7 +8751,7 @@
         </is>
       </c>
       <c r="E78" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0027</v>
       </c>
       <c r="F78" s="2" t="inlineStr">
         <is>
@@ -8781,7 +8781,7 @@
         </is>
       </c>
       <c r="E79" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0038</v>
       </c>
       <c r="F79" s="2" t="inlineStr">
         <is>
@@ -8811,7 +8811,7 @@
         </is>
       </c>
       <c r="E80" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0025</v>
       </c>
       <c r="F80" s="2" t="inlineStr">
         <is>
@@ -8841,7 +8841,7 @@
         </is>
       </c>
       <c r="E81" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0041</v>
       </c>
       <c r="F81" s="2" t="inlineStr">
         <is>
@@ -8871,7 +8871,7 @@
         </is>
       </c>
       <c r="E82" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.003</v>
       </c>
       <c r="F82" s="2" t="inlineStr">
         <is>
@@ -8901,7 +8901,7 @@
         </is>
       </c>
       <c r="E83" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0033</v>
       </c>
       <c r="F83" s="2" t="inlineStr">
         <is>
@@ -8931,7 +8931,7 @@
         </is>
       </c>
       <c r="E84" s="2" t="n">
-        <v>0.0032</v>
+        <v>0.0026</v>
       </c>
       <c r="F84" s="2" t="inlineStr">
         <is>
@@ -8961,7 +8961,7 @@
         </is>
       </c>
       <c r="E85" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0035</v>
       </c>
       <c r="F85" s="2" t="inlineStr">
         <is>
@@ -8991,7 +8991,7 @@
         </is>
       </c>
       <c r="E86" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0037</v>
       </c>
       <c r="F86" s="2" t="inlineStr">
         <is>
@@ -9021,7 +9021,7 @@
         </is>
       </c>
       <c r="E87" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0035</v>
       </c>
       <c r="F87" s="2" t="inlineStr">
         <is>
@@ -9051,7 +9051,7 @@
         </is>
       </c>
       <c r="E88" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.0028</v>
       </c>
       <c r="F88" s="2" t="inlineStr">
         <is>
@@ -9081,7 +9081,7 @@
         </is>
       </c>
       <c r="E89" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0025</v>
       </c>
       <c r="F89" s="2" t="inlineStr">
         <is>
@@ -9111,7 +9111,7 @@
         </is>
       </c>
       <c r="E90" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0031</v>
       </c>
       <c r="F90" s="2" t="inlineStr">
         <is>
@@ -9141,7 +9141,7 @@
         </is>
       </c>
       <c r="E91" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0025</v>
       </c>
       <c r="F91" s="2" t="inlineStr">
         <is>
@@ -9171,7 +9171,7 @@
         </is>
       </c>
       <c r="E92" s="2" t="n">
-        <v>0.0035</v>
+        <v>0.0025</v>
       </c>
       <c r="F92" s="2" t="inlineStr">
         <is>
@@ -9201,7 +9201,7 @@
         </is>
       </c>
       <c r="E93" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0043</v>
       </c>
       <c r="F93" s="2" t="inlineStr">
         <is>
@@ -9231,7 +9231,7 @@
         </is>
       </c>
       <c r="E94" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0023</v>
       </c>
       <c r="F94" s="2" t="inlineStr">
         <is>
@@ -9261,7 +9261,7 @@
         </is>
       </c>
       <c r="E95" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0033</v>
       </c>
       <c r="F95" s="2" t="inlineStr">
         <is>
@@ -9291,7 +9291,7 @@
         </is>
       </c>
       <c r="E96" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0039</v>
       </c>
       <c r="F96" s="2" t="inlineStr">
         <is>
@@ -9321,7 +9321,7 @@
         </is>
       </c>
       <c r="E97" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0024</v>
       </c>
       <c r="F97" s="2" t="inlineStr">
         <is>
@@ -9351,7 +9351,7 @@
         </is>
       </c>
       <c r="E98" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0032</v>
       </c>
       <c r="F98" s="2" t="inlineStr">
         <is>
@@ -9381,7 +9381,7 @@
         </is>
       </c>
       <c r="E99" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0051</v>
       </c>
       <c r="F99" s="2" t="inlineStr">
         <is>
@@ -9411,7 +9411,7 @@
         </is>
       </c>
       <c r="E100" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0023</v>
       </c>
       <c r="F100" s="2" t="inlineStr">
         <is>
@@ -9441,7 +9441,7 @@
         </is>
       </c>
       <c r="E101" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0023</v>
       </c>
       <c r="F101" s="2" t="inlineStr">
         <is>
@@ -9471,7 +9471,7 @@
         </is>
       </c>
       <c r="E102" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0037</v>
       </c>
       <c r="F102" s="2" t="inlineStr">
         <is>
@@ -9501,7 +9501,7 @@
         </is>
       </c>
       <c r="E103" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0025</v>
       </c>
       <c r="F103" s="2" t="inlineStr">
         <is>
@@ -9531,7 +9531,7 @@
         </is>
       </c>
       <c r="E104" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0027</v>
       </c>
       <c r="F104" s="2" t="inlineStr">
         <is>
@@ -9561,7 +9561,7 @@
         </is>
       </c>
       <c r="E105" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0034</v>
       </c>
       <c r="F105" s="2" t="inlineStr">
         <is>
@@ -9591,7 +9591,7 @@
         </is>
       </c>
       <c r="E106" s="2" t="n">
-        <v>0.0038</v>
+        <v>0.0035</v>
       </c>
       <c r="F106" s="2" t="inlineStr">
         <is>
@@ -9621,7 +9621,7 @@
         </is>
       </c>
       <c r="E107" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0026</v>
       </c>
       <c r="F107" s="2" t="inlineStr">
         <is>
@@ -9651,7 +9651,7 @@
         </is>
       </c>
       <c r="E108" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0032</v>
       </c>
       <c r="F108" s="2" t="inlineStr">
         <is>
@@ -9681,7 +9681,7 @@
         </is>
       </c>
       <c r="E109" s="2" t="n">
-        <v>0.002</v>
+        <v>0.004</v>
       </c>
       <c r="F109" s="2" t="inlineStr">
         <is>
@@ -9711,7 +9711,7 @@
         </is>
       </c>
       <c r="E110" s="2" t="n">
-        <v>0.0028</v>
+        <v>0.0047</v>
       </c>
       <c r="F110" s="2" t="inlineStr">
         <is>
@@ -9741,7 +9741,7 @@
         </is>
       </c>
       <c r="E111" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0038</v>
       </c>
       <c r="F111" s="2" t="inlineStr">
         <is>
@@ -9771,7 +9771,7 @@
         </is>
       </c>
       <c r="E112" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0026</v>
       </c>
       <c r="F112" s="2" t="inlineStr">
         <is>
@@ -9801,7 +9801,7 @@
         </is>
       </c>
       <c r="E113" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0047</v>
       </c>
       <c r="F113" s="2" t="inlineStr">
         <is>
@@ -9831,7 +9831,7 @@
         </is>
       </c>
       <c r="E114" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0039</v>
       </c>
       <c r="F114" s="2" t="inlineStr">
         <is>
@@ -9861,7 +9861,7 @@
         </is>
       </c>
       <c r="E115" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0024</v>
       </c>
       <c r="F115" s="2" t="inlineStr">
         <is>
@@ -9891,7 +9891,7 @@
         </is>
       </c>
       <c r="E116" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0035</v>
       </c>
       <c r="F116" s="2" t="inlineStr">
         <is>
@@ -9921,7 +9921,7 @@
         </is>
       </c>
       <c r="E117" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0035</v>
       </c>
       <c r="F117" s="2" t="inlineStr">
         <is>
@@ -9951,7 +9951,7 @@
         </is>
       </c>
       <c r="E118" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0036</v>
       </c>
       <c r="F118" s="2" t="inlineStr">
         <is>
@@ -9981,7 +9981,7 @@
         </is>
       </c>
       <c r="E119" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0042</v>
       </c>
       <c r="F119" s="2" t="inlineStr">
         <is>
@@ -10011,7 +10011,7 @@
         </is>
       </c>
       <c r="E120" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0042</v>
       </c>
       <c r="F120" s="2" t="inlineStr">
         <is>
@@ -10041,7 +10041,7 @@
         </is>
       </c>
       <c r="E121" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.005</v>
       </c>
       <c r="F121" s="2" t="inlineStr">
         <is>
@@ -10071,7 +10071,7 @@
         </is>
       </c>
       <c r="E122" s="2" t="n">
-        <v>0.0146</v>
+        <v>0.0031</v>
       </c>
       <c r="F122" s="2" t="inlineStr">
         <is>
@@ -10101,7 +10101,7 @@
         </is>
       </c>
       <c r="E123" s="2" t="n">
-        <v>0.0031</v>
+        <v>0.0041</v>
       </c>
       <c r="F123" s="2" t="inlineStr">
         <is>
@@ -10131,7 +10131,7 @@
         </is>
       </c>
       <c r="E124" s="2" t="n">
-        <v>0.0037</v>
+        <v>0.0175</v>
       </c>
       <c r="F124" s="2" t="inlineStr">
         <is>
@@ -10161,7 +10161,7 @@
         </is>
       </c>
       <c r="E125" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0065</v>
       </c>
       <c r="F125" s="2" t="inlineStr">
         <is>
@@ -10191,7 +10191,7 @@
         </is>
       </c>
       <c r="E126" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0034</v>
       </c>
       <c r="F126" s="2" t="inlineStr">
         <is>
@@ -10221,7 +10221,7 @@
         </is>
       </c>
       <c r="E127" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0036</v>
       </c>
       <c r="F127" s="2" t="inlineStr">
         <is>
@@ -10251,7 +10251,7 @@
         </is>
       </c>
       <c r="E128" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0047</v>
       </c>
       <c r="F128" s="2" t="inlineStr">
         <is>
@@ -10281,7 +10281,7 @@
         </is>
       </c>
       <c r="E129" s="2" t="n">
-        <v>0.0024</v>
+        <v>0.0055</v>
       </c>
       <c r="F129" s="2" t="inlineStr">
         <is>
@@ -10311,7 +10311,7 @@
         </is>
       </c>
       <c r="E130" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0076</v>
       </c>
       <c r="F130" s="2" t="inlineStr">
         <is>
@@ -10341,7 +10341,7 @@
         </is>
       </c>
       <c r="E131" s="2" t="n">
-        <v>0.0033</v>
+        <v>0.0044</v>
       </c>
       <c r="F131" s="2" t="inlineStr">
         <is>
@@ -10371,7 +10371,7 @@
         </is>
       </c>
       <c r="E132" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0035</v>
       </c>
       <c r="F132" s="2" t="inlineStr">
         <is>
@@ -10401,7 +10401,7 @@
         </is>
       </c>
       <c r="E133" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0029</v>
       </c>
       <c r="F133" s="2" t="inlineStr">
         <is>
@@ -10431,7 +10431,7 @@
         </is>
       </c>
       <c r="E134" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0055</v>
       </c>
       <c r="F134" s="2" t="inlineStr">
         <is>
@@ -10461,7 +10461,7 @@
         </is>
       </c>
       <c r="E135" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0057</v>
       </c>
       <c r="F135" s="2" t="inlineStr">
         <is>
@@ -10491,7 +10491,7 @@
         </is>
       </c>
       <c r="E136" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0047</v>
       </c>
       <c r="F136" s="2" t="inlineStr">
         <is>
@@ -10521,7 +10521,7 @@
         </is>
       </c>
       <c r="E137" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0029</v>
       </c>
       <c r="F137" s="2" t="inlineStr">
         <is>
@@ -10551,7 +10551,7 @@
         </is>
       </c>
       <c r="E138" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0031</v>
       </c>
       <c r="F138" s="2" t="inlineStr">
         <is>
@@ -10581,7 +10581,7 @@
         </is>
       </c>
       <c r="E139" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0106</v>
       </c>
       <c r="F139" s="2" t="inlineStr">
         <is>
@@ -10611,7 +10611,7 @@
         </is>
       </c>
       <c r="E140" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.004</v>
       </c>
       <c r="F140" s="2" t="inlineStr">
         <is>
@@ -10641,7 +10641,7 @@
         </is>
       </c>
       <c r="E141" s="2" t="n">
-        <v>0.003</v>
+        <v>0.0077</v>
       </c>
       <c r="F141" s="2" t="inlineStr">
         <is>
@@ -10671,7 +10671,7 @@
         </is>
       </c>
       <c r="E142" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0049</v>
       </c>
       <c r="F142" s="2" t="inlineStr">
         <is>
@@ -10701,7 +10701,7 @@
         </is>
       </c>
       <c r="E143" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0073</v>
       </c>
       <c r="F143" s="2" t="inlineStr">
         <is>
@@ -10731,7 +10731,7 @@
         </is>
       </c>
       <c r="E144" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0181</v>
       </c>
       <c r="F144" s="2" t="inlineStr">
         <is>
@@ -10761,7 +10761,7 @@
         </is>
       </c>
       <c r="E145" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.004</v>
       </c>
       <c r="F145" s="2" t="inlineStr">
         <is>
@@ -10791,7 +10791,7 @@
         </is>
       </c>
       <c r="E146" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0048</v>
       </c>
       <c r="F146" s="2" t="inlineStr">
         <is>
@@ -10821,7 +10821,7 @@
         </is>
       </c>
       <c r="E147" s="2" t="n">
-        <v>0.0022</v>
+        <v>0.0043</v>
       </c>
       <c r="F147" s="2" t="inlineStr">
         <is>
@@ -10851,7 +10851,7 @@
         </is>
       </c>
       <c r="E148" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0059</v>
       </c>
       <c r="F148" s="2" t="inlineStr">
         <is>
@@ -10881,7 +10881,7 @@
         </is>
       </c>
       <c r="E149" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0045</v>
       </c>
       <c r="F149" s="2" t="inlineStr">
         <is>
@@ -10911,7 +10911,7 @@
         </is>
       </c>
       <c r="E150" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0042</v>
       </c>
       <c r="F150" s="2" t="inlineStr">
         <is>
@@ -10941,7 +10941,7 @@
         </is>
       </c>
       <c r="E151" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0031</v>
       </c>
       <c r="F151" s="2" t="inlineStr">
         <is>
@@ -10971,7 +10971,7 @@
         </is>
       </c>
       <c r="E152" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0043</v>
       </c>
       <c r="F152" s="2" t="inlineStr">
         <is>
@@ -11001,7 +11001,7 @@
         </is>
       </c>
       <c r="E153" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0026</v>
       </c>
       <c r="F153" s="2" t="inlineStr">
         <is>
@@ -11031,7 +11031,7 @@
         </is>
       </c>
       <c r="E154" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0027</v>
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
@@ -11061,7 +11061,7 @@
         </is>
       </c>
       <c r="E155" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0053</v>
       </c>
       <c r="F155" s="2" t="inlineStr">
         <is>
@@ -11091,7 +11091,7 @@
         </is>
       </c>
       <c r="E156" s="2" t="n">
-        <v>0.0029</v>
+        <v>0.0031</v>
       </c>
       <c r="F156" s="2" t="inlineStr">
         <is>
@@ -11121,7 +11121,7 @@
         </is>
       </c>
       <c r="E157" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0031</v>
       </c>
       <c r="F157" s="2" t="inlineStr">
         <is>
@@ -11151,7 +11151,7 @@
         </is>
       </c>
       <c r="E158" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0043</v>
       </c>
       <c r="F158" s="2" t="inlineStr">
         <is>
@@ -11181,7 +11181,7 @@
         </is>
       </c>
       <c r="E159" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0045</v>
       </c>
       <c r="F159" s="2" t="inlineStr">
         <is>
@@ -11211,7 +11211,7 @@
         </is>
       </c>
       <c r="E160" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0035</v>
       </c>
       <c r="F160" s="2" t="inlineStr">
         <is>
@@ -11241,7 +11241,7 @@
         </is>
       </c>
       <c r="E161" s="2" t="n">
-        <v>0.0036</v>
+        <v>0.0027</v>
       </c>
       <c r="F161" s="2" t="inlineStr">
         <is>
@@ -11271,7 +11271,7 @@
         </is>
       </c>
       <c r="E162" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F162" s="2" t="inlineStr">
         <is>
@@ -11301,7 +11301,7 @@
         </is>
       </c>
       <c r="E163" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0021</v>
       </c>
       <c r="F163" s="2" t="inlineStr">
         <is>
@@ -11331,7 +11331,7 @@
         </is>
       </c>
       <c r="E164" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0013</v>
       </c>
       <c r="F164" s="2" t="inlineStr">
         <is>
@@ -11361,7 +11361,7 @@
         </is>
       </c>
       <c r="E165" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.0027</v>
       </c>
       <c r="F165" s="2" t="inlineStr">
         <is>
@@ -11391,7 +11391,7 @@
         </is>
       </c>
       <c r="E166" s="2" t="n">
-        <v>0.0008</v>
+        <v>0.002</v>
       </c>
       <c r="F166" s="2" t="inlineStr">
         <is>
@@ -11421,7 +11421,7 @@
         </is>
       </c>
       <c r="E167" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0017</v>
       </c>
       <c r="F167" s="2" t="inlineStr">
         <is>
@@ -11451,7 +11451,7 @@
         </is>
       </c>
       <c r="E168" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0022</v>
       </c>
       <c r="F168" s="2" t="inlineStr">
         <is>
@@ -11481,7 +11481,7 @@
         </is>
       </c>
       <c r="E169" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0023</v>
       </c>
       <c r="F169" s="2" t="inlineStr">
         <is>
@@ -11511,7 +11511,7 @@
         </is>
       </c>
       <c r="E170" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0041</v>
       </c>
       <c r="F170" s="2" t="inlineStr">
         <is>
@@ -11541,7 +11541,7 @@
         </is>
       </c>
       <c r="E171" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0065</v>
       </c>
       <c r="F171" s="2" t="inlineStr">
         <is>
@@ -11571,7 +11571,7 @@
         </is>
       </c>
       <c r="E172" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0038</v>
       </c>
       <c r="F172" s="2" t="inlineStr">
         <is>
@@ -11601,7 +11601,7 @@
         </is>
       </c>
       <c r="E173" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0053</v>
       </c>
       <c r="F173" s="2" t="inlineStr">
         <is>
@@ -11631,7 +11631,7 @@
         </is>
       </c>
       <c r="E174" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0037</v>
       </c>
       <c r="F174" s="2" t="inlineStr">
         <is>
@@ -11661,7 +11661,7 @@
         </is>
       </c>
       <c r="E175" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0017</v>
       </c>
       <c r="F175" s="2" t="inlineStr">
         <is>
@@ -11691,7 +11691,7 @@
         </is>
       </c>
       <c r="E176" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.003</v>
       </c>
       <c r="F176" s="2" t="inlineStr">
         <is>
@@ -11721,7 +11721,7 @@
         </is>
       </c>
       <c r="E177" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0016</v>
       </c>
       <c r="F177" s="2" t="inlineStr">
         <is>
@@ -11751,7 +11751,7 @@
         </is>
       </c>
       <c r="E178" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0025</v>
       </c>
       <c r="F178" s="2" t="inlineStr">
         <is>
@@ -11781,7 +11781,7 @@
         </is>
       </c>
       <c r="E179" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F179" s="2" t="inlineStr">
         <is>
@@ -11811,7 +11811,7 @@
         </is>
       </c>
       <c r="E180" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0026</v>
       </c>
       <c r="F180" s="2" t="inlineStr">
         <is>
@@ -11841,7 +11841,7 @@
         </is>
       </c>
       <c r="E181" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0033</v>
       </c>
       <c r="F181" s="2" t="inlineStr">
         <is>
@@ -11871,7 +11871,7 @@
         </is>
       </c>
       <c r="E182" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0024</v>
       </c>
       <c r="F182" s="2" t="inlineStr">
         <is>
@@ -11901,7 +11901,7 @@
         </is>
       </c>
       <c r="E183" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0027</v>
       </c>
       <c r="F183" s="2" t="inlineStr">
         <is>
@@ -11931,7 +11931,7 @@
         </is>
       </c>
       <c r="E184" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0014</v>
       </c>
       <c r="F184" s="2" t="inlineStr">
         <is>
@@ -11961,7 +11961,7 @@
         </is>
       </c>
       <c r="E185" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0024</v>
       </c>
       <c r="F185" s="2" t="inlineStr">
         <is>
@@ -11991,7 +11991,7 @@
         </is>
       </c>
       <c r="E186" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0021</v>
       </c>
       <c r="F186" s="2" t="inlineStr">
         <is>
@@ -12021,7 +12021,7 @@
         </is>
       </c>
       <c r="E187" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0024</v>
       </c>
       <c r="F187" s="2" t="inlineStr">
         <is>
@@ -12051,7 +12051,7 @@
         </is>
       </c>
       <c r="E188" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0028</v>
       </c>
       <c r="F188" s="2" t="inlineStr">
         <is>
@@ -12081,7 +12081,7 @@
         </is>
       </c>
       <c r="E189" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0032</v>
       </c>
       <c r="F189" s="2" t="inlineStr">
         <is>
@@ -12111,7 +12111,7 @@
         </is>
       </c>
       <c r="E190" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0027</v>
       </c>
       <c r="F190" s="2" t="inlineStr">
         <is>
@@ -12141,7 +12141,7 @@
         </is>
       </c>
       <c r="E191" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0026</v>
       </c>
       <c r="F191" s="2" t="inlineStr">
         <is>
@@ -12171,7 +12171,7 @@
         </is>
       </c>
       <c r="E192" s="2" t="n">
-        <v>0.0023</v>
+        <v>0.0046</v>
       </c>
       <c r="F192" s="2" t="inlineStr">
         <is>
@@ -12201,7 +12201,7 @@
         </is>
       </c>
       <c r="E193" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0046</v>
       </c>
       <c r="F193" s="2" t="inlineStr">
         <is>
@@ -12231,7 +12231,7 @@
         </is>
       </c>
       <c r="E194" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0047</v>
       </c>
       <c r="F194" s="2" t="inlineStr">
         <is>
@@ -12261,7 +12261,7 @@
         </is>
       </c>
       <c r="E195" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0028</v>
       </c>
       <c r="F195" s="2" t="inlineStr">
         <is>
@@ -12291,7 +12291,7 @@
         </is>
       </c>
       <c r="E196" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0041</v>
       </c>
       <c r="F196" s="2" t="inlineStr">
         <is>
@@ -12321,7 +12321,7 @@
         </is>
       </c>
       <c r="E197" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0029</v>
       </c>
       <c r="F197" s="2" t="inlineStr">
         <is>
@@ -12351,7 +12351,7 @@
         </is>
       </c>
       <c r="E198" s="2" t="n">
-        <v>0.0027</v>
+        <v>0.0054</v>
       </c>
       <c r="F198" s="2" t="inlineStr">
         <is>
@@ -12381,7 +12381,7 @@
         </is>
       </c>
       <c r="E199" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0047</v>
       </c>
       <c r="F199" s="2" t="inlineStr">
         <is>
@@ -12411,7 +12411,7 @@
         </is>
       </c>
       <c r="E200" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0039</v>
       </c>
       <c r="F200" s="2" t="inlineStr">
         <is>
@@ -12441,7 +12441,7 @@
         </is>
       </c>
       <c r="E201" s="2" t="n">
-        <v>0.0026</v>
+        <v>0.0053</v>
       </c>
       <c r="F201" s="2" t="inlineStr">
         <is>
@@ -12471,7 +12471,7 @@
         </is>
       </c>
       <c r="E202" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0023</v>
       </c>
       <c r="F202" s="2" t="inlineStr">
         <is>
@@ -12501,7 +12501,7 @@
         </is>
       </c>
       <c r="E203" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0028</v>
       </c>
       <c r="F203" s="2" t="inlineStr">
         <is>
@@ -12531,7 +12531,7 @@
         </is>
       </c>
       <c r="E204" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0032</v>
       </c>
       <c r="F204" s="2" t="inlineStr">
         <is>
@@ -12561,7 +12561,7 @@
         </is>
       </c>
       <c r="E205" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0026</v>
       </c>
       <c r="F205" s="2" t="inlineStr">
         <is>
@@ -12591,7 +12591,7 @@
         </is>
       </c>
       <c r="E206" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0027</v>
       </c>
       <c r="F206" s="2" t="inlineStr">
         <is>
@@ -12621,7 +12621,7 @@
         </is>
       </c>
       <c r="E207" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0019</v>
       </c>
       <c r="F207" s="2" t="inlineStr">
         <is>
@@ -12651,7 +12651,7 @@
         </is>
       </c>
       <c r="E208" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0037</v>
       </c>
       <c r="F208" s="2" t="inlineStr">
         <is>
@@ -12681,7 +12681,7 @@
         </is>
       </c>
       <c r="E209" s="2" t="n">
-        <v>0.0025</v>
+        <v>0.0055</v>
       </c>
       <c r="F209" s="2" t="inlineStr">
         <is>
@@ -12711,7 +12711,7 @@
         </is>
       </c>
       <c r="E210" s="2" t="n">
-        <v>0.002</v>
+        <v>0.0036</v>
       </c>
       <c r="F210" s="2" t="inlineStr">
         <is>
@@ -12741,7 +12741,7 @@
         </is>
       </c>
       <c r="E211" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0023</v>
       </c>
       <c r="F211" s="2" t="inlineStr">
         <is>
@@ -12771,7 +12771,7 @@
         </is>
       </c>
       <c r="E212" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0019</v>
       </c>
       <c r="F212" s="2" t="inlineStr">
         <is>
@@ -12801,7 +12801,7 @@
         </is>
       </c>
       <c r="E213" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0017</v>
       </c>
       <c r="F213" s="2" t="inlineStr">
         <is>
@@ -12831,7 +12831,7 @@
         </is>
       </c>
       <c r="E214" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.002</v>
       </c>
       <c r="F214" s="2" t="inlineStr">
         <is>
@@ -12861,7 +12861,7 @@
         </is>
       </c>
       <c r="E215" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0016</v>
       </c>
       <c r="F215" s="2" t="inlineStr">
         <is>
@@ -12891,7 +12891,7 @@
         </is>
       </c>
       <c r="E216" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0018</v>
       </c>
       <c r="F216" s="2" t="inlineStr">
         <is>
@@ -12921,7 +12921,7 @@
         </is>
       </c>
       <c r="E217" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0027</v>
       </c>
       <c r="F217" s="2" t="inlineStr">
         <is>
@@ -12951,7 +12951,7 @@
         </is>
       </c>
       <c r="E218" s="2" t="n">
-        <v>0.0019</v>
+        <v>0.0032</v>
       </c>
       <c r="F218" s="2" t="inlineStr">
         <is>
@@ -12981,7 +12981,7 @@
         </is>
       </c>
       <c r="E219" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0028</v>
       </c>
       <c r="F219" s="2" t="inlineStr">
         <is>
@@ -13011,7 +13011,7 @@
         </is>
       </c>
       <c r="E220" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0021</v>
       </c>
       <c r="F220" s="2" t="inlineStr">
         <is>
@@ -13041,7 +13041,7 @@
         </is>
       </c>
       <c r="E221" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0023</v>
       </c>
       <c r="F221" s="2" t="inlineStr">
         <is>
@@ -13071,7 +13071,7 @@
         </is>
       </c>
       <c r="E222" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0032</v>
       </c>
       <c r="F222" s="2" t="inlineStr">
         <is>
@@ -13131,7 +13131,7 @@
         </is>
       </c>
       <c r="E224" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0032</v>
       </c>
       <c r="F224" s="2" t="inlineStr">
         <is>
@@ -13161,7 +13161,7 @@
         </is>
       </c>
       <c r="E225" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0035</v>
       </c>
       <c r="F225" s="2" t="inlineStr">
         <is>
@@ -13191,7 +13191,7 @@
         </is>
       </c>
       <c r="E226" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0021</v>
       </c>
       <c r="F226" s="2" t="inlineStr">
         <is>
@@ -13221,7 +13221,7 @@
         </is>
       </c>
       <c r="E227" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0025</v>
       </c>
       <c r="F227" s="2" t="inlineStr">
         <is>
@@ -13251,7 +13251,7 @@
         </is>
       </c>
       <c r="E228" s="2" t="n">
-        <v>0.001</v>
+        <v>0.015</v>
       </c>
       <c r="F228" s="2" t="inlineStr">
         <is>
@@ -13281,7 +13281,7 @@
         </is>
       </c>
       <c r="E229" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0017</v>
       </c>
       <c r="F229" s="2" t="inlineStr">
         <is>
@@ -13311,7 +13311,7 @@
         </is>
       </c>
       <c r="E230" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0025</v>
       </c>
       <c r="F230" s="2" t="inlineStr">
         <is>
@@ -13341,7 +13341,7 @@
         </is>
       </c>
       <c r="E231" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0023</v>
       </c>
       <c r="F231" s="2" t="inlineStr">
         <is>
@@ -13371,7 +13371,7 @@
         </is>
       </c>
       <c r="E232" s="2" t="n">
-        <v>0.0021</v>
+        <v>0.0029</v>
       </c>
       <c r="F232" s="2" t="inlineStr">
         <is>
@@ -13401,7 +13401,7 @@
         </is>
       </c>
       <c r="E233" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0015</v>
       </c>
       <c r="F233" s="2" t="inlineStr">
         <is>
@@ -13431,7 +13431,7 @@
         </is>
       </c>
       <c r="E234" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0015</v>
       </c>
       <c r="F234" s="2" t="inlineStr">
         <is>
@@ -13461,7 +13461,7 @@
         </is>
       </c>
       <c r="E235" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0015</v>
       </c>
       <c r="F235" s="2" t="inlineStr">
         <is>
@@ -13491,7 +13491,7 @@
         </is>
       </c>
       <c r="E236" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0011</v>
       </c>
       <c r="F236" s="2" t="inlineStr">
         <is>
@@ -13521,7 +13521,7 @@
         </is>
       </c>
       <c r="E237" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0013</v>
       </c>
       <c r="F237" s="2" t="inlineStr">
         <is>
@@ -13551,7 +13551,7 @@
         </is>
       </c>
       <c r="E238" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.0016</v>
       </c>
       <c r="F238" s="2" t="inlineStr">
         <is>
@@ -13581,7 +13581,7 @@
         </is>
       </c>
       <c r="E239" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0015</v>
       </c>
       <c r="F239" s="2" t="inlineStr">
         <is>
@@ -13611,7 +13611,7 @@
         </is>
       </c>
       <c r="E240" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0012</v>
       </c>
       <c r="F240" s="2" t="inlineStr">
         <is>
@@ -13641,7 +13641,7 @@
         </is>
       </c>
       <c r="E241" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0014</v>
       </c>
       <c r="F241" s="2" t="inlineStr">
         <is>
@@ -13671,7 +13671,7 @@
         </is>
       </c>
       <c r="E242" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0013</v>
       </c>
       <c r="F242" s="2" t="inlineStr">
         <is>
@@ -13701,7 +13701,7 @@
         </is>
       </c>
       <c r="E243" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0014</v>
       </c>
       <c r="F243" s="2" t="inlineStr">
         <is>
@@ -13731,7 +13731,7 @@
         </is>
       </c>
       <c r="E244" s="2" t="n">
-        <v>0.0014</v>
+        <v>0.0017</v>
       </c>
       <c r="F244" s="2" t="inlineStr">
         <is>
@@ -13761,7 +13761,7 @@
         </is>
       </c>
       <c r="E245" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0019</v>
       </c>
       <c r="F245" s="2" t="inlineStr">
         <is>
@@ -13791,7 +13791,7 @@
         </is>
       </c>
       <c r="E246" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0017</v>
       </c>
       <c r="F246" s="2" t="inlineStr">
         <is>
@@ -13821,7 +13821,7 @@
         </is>
       </c>
       <c r="E247" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0012</v>
       </c>
       <c r="F247" s="2" t="inlineStr">
         <is>
@@ -13851,7 +13851,7 @@
         </is>
       </c>
       <c r="E248" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0014</v>
       </c>
       <c r="F248" s="2" t="inlineStr">
         <is>
@@ -13881,7 +13881,7 @@
         </is>
       </c>
       <c r="E249" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0012</v>
       </c>
       <c r="F249" s="2" t="inlineStr">
         <is>
@@ -13911,7 +13911,7 @@
         </is>
       </c>
       <c r="E250" s="2" t="n">
-        <v>0.0016</v>
+        <v>0.0012</v>
       </c>
       <c r="F250" s="2" t="inlineStr">
         <is>
@@ -13941,7 +13941,7 @@
         </is>
       </c>
       <c r="E251" s="2" t="n">
-        <v>0.0015</v>
+        <v>0.0022</v>
       </c>
       <c r="F251" s="2" t="inlineStr">
         <is>
@@ -13971,7 +13971,7 @@
         </is>
       </c>
       <c r="E252" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0016</v>
       </c>
       <c r="F252" s="2" t="inlineStr">
         <is>
@@ -14001,7 +14001,7 @@
         </is>
       </c>
       <c r="E253" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.0012</v>
       </c>
       <c r="F253" s="2" t="inlineStr">
         <is>
@@ -14031,7 +14031,7 @@
         </is>
       </c>
       <c r="E254" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F254" s="2" t="inlineStr">
         <is>
@@ -14061,7 +14061,7 @@
         </is>
       </c>
       <c r="E255" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F255" s="2" t="inlineStr">
         <is>
@@ -14091,7 +14091,7 @@
         </is>
       </c>
       <c r="E256" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F256" s="2" t="inlineStr">
         <is>
@@ -14121,7 +14121,7 @@
         </is>
       </c>
       <c r="E257" s="2" t="n">
-        <v>0.0017</v>
+        <v>0.0012</v>
       </c>
       <c r="F257" s="2" t="inlineStr">
         <is>
@@ -14151,7 +14151,7 @@
         </is>
       </c>
       <c r="E258" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0014</v>
       </c>
       <c r="F258" s="2" t="inlineStr">
         <is>
@@ -14181,7 +14181,7 @@
         </is>
       </c>
       <c r="E259" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0015</v>
       </c>
       <c r="F259" s="2" t="inlineStr">
         <is>
@@ -14211,7 +14211,7 @@
         </is>
       </c>
       <c r="E260" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0029</v>
       </c>
       <c r="F260" s="2" t="inlineStr">
         <is>
@@ -14241,7 +14241,7 @@
         </is>
       </c>
       <c r="E261" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F261" s="2" t="inlineStr">
         <is>
@@ -14271,7 +14271,7 @@
         </is>
       </c>
       <c r="E262" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0013</v>
       </c>
       <c r="F262" s="2" t="inlineStr">
         <is>
@@ -14301,7 +14301,7 @@
         </is>
       </c>
       <c r="E263" s="2" t="n">
-        <v>0.0009</v>
+        <v>0.013</v>
       </c>
       <c r="F263" s="2" t="inlineStr">
         <is>
@@ -14331,7 +14331,7 @@
         </is>
       </c>
       <c r="E264" s="2" t="n">
-        <v>0.0012</v>
+        <v>0.0014</v>
       </c>
       <c r="F264" s="2" t="inlineStr">
         <is>
@@ -14361,7 +14361,7 @@
         </is>
       </c>
       <c r="E265" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.002</v>
       </c>
       <c r="F265" s="2" t="inlineStr">
         <is>
@@ -14391,7 +14391,7 @@
         </is>
       </c>
       <c r="E266" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0025</v>
       </c>
       <c r="F266" s="2" t="inlineStr">
         <is>
@@ -14421,7 +14421,7 @@
         </is>
       </c>
       <c r="E267" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0014</v>
       </c>
       <c r="F267" s="2" t="inlineStr">
         <is>
@@ -14451,7 +14451,7 @@
         </is>
       </c>
       <c r="E268" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.0014</v>
       </c>
       <c r="F268" s="2" t="inlineStr">
         <is>
@@ -14481,7 +14481,7 @@
         </is>
       </c>
       <c r="E269" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0016</v>
       </c>
       <c r="F269" s="2" t="inlineStr">
         <is>
@@ -14511,7 +14511,7 @@
         </is>
       </c>
       <c r="E270" s="2" t="n">
-        <v>0.0018</v>
+        <v>0.003</v>
       </c>
       <c r="F270" s="2" t="inlineStr">
         <is>
@@ -14541,7 +14541,7 @@
         </is>
       </c>
       <c r="E271" s="2" t="n">
-        <v>0.0011</v>
+        <v>0.002</v>
       </c>
       <c r="F271" s="2" t="inlineStr">
         <is>
@@ -14571,7 +14571,7 @@
         </is>
       </c>
       <c r="E272" s="2" t="n">
-        <v>0.001</v>
+        <v>0.0015</v>
       </c>
       <c r="F272" s="2" t="inlineStr">
         <is>
@@ -14601,7 +14601,7 @@
         </is>
       </c>
       <c r="E273" s="2" t="n">
-        <v>0.001</v>
+        <v>0.002</v>
       </c>
       <c r="F273" s="2" t="inlineStr">
         <is>

</xml_diff>